<commit_message>
Add AI extraction approach using Ollama
- Add PdfExtractor base class shared by rule-based and AI extractors
- Add AiPdfExtractor (pdfplumber + Ollama) with prompt template
- Add Extraction Approach selection to the GUI
- Store quantity as integer in both approaches

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/samples/XLSX_files/extracted_pdf-expected1.xlsx
+++ b/tests/samples/XLSX_files/extracted_pdf-expected1.xlsx
@@ -464,10 +464,8 @@
           <t>Cover, Plastic, MSFD Alarm PCB</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C2" t="n">
+        <v>3</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -491,10 +489,8 @@
           <t>Cover, Plastic, MSFD Voltage M</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C3" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -518,10 +514,8 @@
           <t>Bracket, Back Divider CPRI 1U 19”</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C4" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -545,10 +539,8 @@
           <t>Bracket, Step, 12 Position, Neutral</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
+      <c r="C5" t="n">
+        <v>30</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -572,10 +564,8 @@
           <t>Cover Asm, Top, 3-Pos 1U Alarm RM</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="C6" t="n">
+        <v>100</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -599,10 +589,8 @@
           <t>Bracket, Mounting, Universal YH/YQ-ZH/ZQ</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
+      <c r="C7" t="n">
+        <v>61</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -626,10 +614,8 @@
           <t>Harness, 3 Chan Strikesorb Alarm</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="C8" t="n">
+        <v>50</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -653,10 +639,8 @@
           <t>Busbar, GND A Box GEN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+      <c r="C9" t="n">
+        <v>20</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -680,10 +664,8 @@
           <t>Busbar, Ground, GB3-3-00-X</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="C10" t="n">
+        <v>50</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -707,10 +689,8 @@
           <t>Busbar, Bridge, 7 Pos, 26mm Pitch, L1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
+      <c r="C11" t="n">
+        <v>60</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -734,10 +714,8 @@
           <t>Busbar, Return, Strikesorb 30, AL</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>145</t>
-        </is>
+      <c r="C12" t="n">
+        <v>145</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -761,10 +739,8 @@
           <t>Bus Bar, Neutral, RMx-ED</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+      <c r="C13" t="n">
+        <v>23</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -788,10 +764,8 @@
           <t>Encl, RBMDC-1113-BDU-48 Cover</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C14" t="n">
+        <v>35</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -815,10 +789,8 @@
           <t>Encl, RBMDC-1113-BDU-48 Rear Cover</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="C15" t="n">
+        <v>34</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -842,10 +814,8 @@
           <t>Encl, RBMDC-1113-BDU-48 PSM Cover</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C16" t="n">
+        <v>35</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -869,10 +839,8 @@
           <t>Encl, RBMDC-1113-BDU-48 Front Cover</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C17" t="n">
+        <v>35</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -896,10 +864,8 @@
           <t>Bus Bar, BDU, Front Input, Supply</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C18" t="n">
+        <v>35</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -923,10 +889,8 @@
           <t>Bus Bar, BDU, Front Input, Return</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C19" t="n">
+        <v>35</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -950,10 +914,8 @@
           <t>Bus Bar, BDU, Front Input, Ground</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C20" t="n">
+        <v>35</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -977,10 +939,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, -48V, Input</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
+      <c r="C21" t="n">
+        <v>18</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1004,10 +964,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, RTN</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C22" t="n">
+        <v>35</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1031,10 +989,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, RTN, Input</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+      <c r="C23" t="n">
+        <v>29</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1058,10 +1014,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, GND, Input</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C24" t="n">
+        <v>35</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1085,10 +1039,8 @@
           <t>Bus Bar, BDU Breaker Supply, 16 Pos</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C25" t="n">
+        <v>4</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1112,10 +1064,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, -48V</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>559</t>
-        </is>
+      <c r="C26" t="n">
+        <v>559</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1139,10 +1089,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, PSM -48V/RTN</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>70</t>
-        </is>
+      <c r="C27" t="n">
+        <v>70</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1166,10 +1114,8 @@
           <t>Bus Bar, RBMDC-1113-BDU-48, PSM GND</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
+      <c r="C28" t="n">
+        <v>34</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1193,10 +1139,8 @@
           <t>Bus Bar, BDU, PSM Base, Rear Ground, Alt</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
+      <c r="C29" t="n">
+        <v>35</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1220,10 +1164,8 @@
           <t>PCB Cover</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>330</t>
-        </is>
+      <c r="C30" t="n">
+        <v>330</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1247,10 +1189,8 @@
           <t>Encl, 18.5x8.84, N4, SS, Ltch, KO,Bl,BK</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C31" t="n">
+        <v>3</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1274,10 +1214,8 @@
           <t>Shield, EMI, RSE-2 Indication PCB</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="C32" t="n">
+        <v>50</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1301,10 +1239,8 @@
           <t>Encl, Cover Tray 2, RTF-1502</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C33" t="n">
+        <v>1</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1328,10 +1264,8 @@
           <t>Encl, 14x9x5, Cont Hinge, NEMA 4, SS</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C34" t="n">
+        <v>1</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1355,10 +1289,8 @@
           <t>Bracket, Rectifier Slider, AiO Single</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="C35" t="n">
+        <v>5</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1382,10 +1314,8 @@
           <t>Busbar, GND A Box GEN</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+      <c r="C36" t="n">
+        <v>50</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1409,10 +1339,8 @@
           <t>Busbar, Bridge, 8 Pos, 26mm Pitch</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
+      <c r="C37" t="n">
+        <v>300</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1436,10 +1364,8 @@
           <t>Encl, 10x10x6, 9E Series, EGS</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C38" t="n">
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1463,10 +1389,8 @@
           <t>Bracket, Mounting,Universal RSD</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="C39" t="n">
+        <v>150</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1490,10 +1414,8 @@
           <t>Busbar, DIN, Strikesorb Neutral Mt w/Lug</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
+      <c r="C40" t="n">
+        <v>200</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>

</xml_diff>